<commit_message>
🕒 Auto update: LeetCode data at 2025-11-04 19:10:28 UTC
</commit_message>
<xml_diff>
--- a/leetcode_data.xlsx
+++ b/leetcode_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>Timestamp</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -475,6 +480,7 @@
           <t>2025-11-04 19:00:14</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -496,6 +502,7 @@
           <t>2025-11-04 19:00:14</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -517,6 +524,7 @@
           <t>2025-11-04 19:00:14</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -537,6 +545,55 @@
         <is>
           <t>2025-11-04 19:00:14</t>
         </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>aayanv5201</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2025-11-04 19:10:23</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Santhosh2005</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2025-11-04 19:10:26</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🕒 Auto update: LeetCode data at 2025-11-04 19:11:37 UTC
</commit_message>
<xml_diff>
--- a/leetcode_data.xlsx
+++ b/leetcode_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,6 +596,54 @@
         <v>5</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>aayanv5201</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2025-11-04 19:11:33</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Santhosh2005</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2025-11-04 19:11:35</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🕒 Auto update: LeetCode data at 2025-11-04 19:26:10 UTC
</commit_message>
<xml_diff>
--- a/leetcode_data.xlsx
+++ b/leetcode_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,54 @@
         <v>5</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>aayanv5201</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2025-11-04 19:26:04</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Santhosh2005</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2025-11-04 19:26:08</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>